<commit_message>
docs(template): 단체 신청 양식 ZIP 사진 PNG 안내 추가
- 대학교 학생증·일반카드 양식 작성안내 ZIP 구조에 신청자 사진은 PNG로 준비하도록 명시

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/bulk-excel-templates-20260818/대학교_학생증_단체신청_양식_v1.2.xlsx
+++ b/outputs/bulk-excel-templates-20260818/대학교_학생증_단체신청_양식_v1.2.xlsx
@@ -3365,7 +3365,7 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>로고와 직인은 ZIP에 넣지 않고 신청 화면의 별도 파일 입력에서 업로드합니다.</t>
+          <t>웹 신청 화면에서 학교(학교 검색)와 카드 방향(가로형/세로형)을 먼저 선택해야 합니다. 선택한 방향에 맞는 디자인으로 카드가 만들어집니다. 로고와 직인은 ZIP에 넣지 않고 신청 화면의 별도 파일 입력에서 업로드합니다.</t>
         </is>
       </c>
     </row>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>유효한 이메일을 입력합니다. 서버에서 앞뒤 공백을 제거하고 소문자로 정규화합니다.</t>
+          <t>모든 신청자의 이메일을 빠짐없이, 정확한 형식으로 입력해 주세요. 이메일이 없거나 잘못 적히면 발급된 카드 이미지를 내려받기 어려울 수 있습니다.</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>ZIP 루트에 .xlsx 파일 정확히 1개와 신청자 사진을 둡니다. __MACOSX와 .DS_Store는 무시되지만 하위 폴더 파일은 사진으로 인정하지 않습니다.</t>
+          <t>ZIP 루트에 .xlsx 파일 정확히 1개와 신청자 사진을 둡니다. __MACOSX와 .DS_Store는 무시되지만 하위 폴더 파일은 사진으로 인정하지 않습니다. 신청자 사진은 반드시 PNG(.png) 파일로 준비해 주세요. JPG 등 다른 형식은 사용할 수 없습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>